<commit_message>
Allow resizing columns/rows in locked Excel templates
Sheet protection was blocking column and row resizing by default
(Excel's standard lockdown), which meant a cell with long text made
the next column's content unreadable without clicking into it, with
no way to widen the previous column to compensate. Resizing is purely
cosmetic - it doesn't let anyone write outside the authorized cells or
touch the data validation - so it's now explicitly allowed while
everything else (inserting/deleting rows/columns, reformatting cell
content, sheet/workbook structure) stays locked.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/data/excel_templates/organizations.xlsx
+++ b/apps/api/data/excel_templates/organizations.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_lists" sheetId="2" state="veryHidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'organizations'!$A$1:$Y$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'organizations'!$A$1:$AE$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -57,18 +57,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,34 +432,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:AE1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" style="5" min="1" max="1"/>
-    <col width="18" customWidth="1" style="5" min="2" max="2"/>
-    <col width="18" customWidth="1" style="5" min="3" max="3"/>
+    <col width="18" customWidth="1" style="1" min="1" max="1"/>
+    <col width="18" customWidth="1" style="1" min="2" max="2"/>
+    <col width="18" customWidth="1" style="1" min="3" max="3"/>
     <col width="18" customWidth="1" style="1" min="4" max="4"/>
     <col width="18" customWidth="1" style="1" min="5" max="5"/>
-    <col width="18" customWidth="1" style="5" min="6" max="6"/>
-    <col width="18" customWidth="1" style="5" min="7" max="7"/>
-    <col width="18" customWidth="1" style="5" min="8" max="8"/>
-    <col width="18" customWidth="1" style="1" min="9" max="9"/>
-    <col width="18" customWidth="1" style="5" min="10" max="10"/>
-    <col width="18" customWidth="1" style="5" min="11" max="11"/>
-    <col width="18" customWidth="1" style="5" min="12" max="12"/>
-    <col width="18" customWidth="1" style="5" min="13" max="13"/>
+    <col width="18" customWidth="1" style="1" min="6" max="6"/>
+    <col width="18" customWidth="1" style="1" min="7" max="7"/>
+    <col width="18" customWidth="1" style="1" min="8" max="8"/>
+    <col width="23" customWidth="1" style="1" min="9" max="9"/>
+    <col width="18" customWidth="1" style="1" min="10" max="10"/>
+    <col width="18" customWidth="1" style="1" min="11" max="11"/>
+    <col width="18" customWidth="1" style="1" min="12" max="12"/>
+    <col width="18" customWidth="1" style="1" min="13" max="13"/>
     <col width="18" customWidth="1" style="1" min="14" max="14"/>
-    <col width="18" customWidth="1" style="5" min="15" max="15"/>
-    <col width="18" customWidth="1" style="5" min="16" max="16"/>
+    <col width="18" customWidth="1" style="1" min="15" max="15"/>
+    <col width="18" customWidth="1" style="1" min="16" max="16"/>
     <col width="18" customWidth="1" style="1" min="17" max="17"/>
     <col width="18" customWidth="1" style="1" min="18" max="18"/>
-    <col width="18" customWidth="1" style="6" min="19" max="19"/>
-    <col width="18" customWidth="1" style="5" min="20" max="20"/>
-    <col width="21" customWidth="1" style="5" min="21" max="21"/>
-    <col width="18" customWidth="1" style="6" min="22" max="22"/>
-    <col width="24" customWidth="1" style="6" min="23" max="23"/>
-    <col width="26" customWidth="1" style="5" min="24" max="24"/>
-    <col width="18" customWidth="1" style="5" min="25" max="25"/>
+    <col width="18" customWidth="1" style="1" min="19" max="19"/>
+    <col width="18" customWidth="1" style="1" min="20" max="20"/>
+    <col width="18" customWidth="1" style="2" min="21" max="21"/>
+    <col width="18" customWidth="1" style="1" min="22" max="22"/>
+    <col width="18" customWidth="1" style="1" min="23" max="23"/>
+    <col width="18" customWidth="1" style="1" min="24" max="24"/>
+    <col width="18" customWidth="1" style="2" min="25" max="25"/>
+    <col width="18" customWidth="1" style="1" min="26" max="26"/>
+    <col width="21" customWidth="1" style="1" min="27" max="27"/>
+    <col width="18" customWidth="1" style="2" min="28" max="28"/>
+    <col width="24" customWidth="1" style="2" min="29" max="29"/>
+    <col width="26" customWidth="1" style="1" min="30" max="30"/>
+    <col width="18" customWidth="1" style="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,12 +486,12 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>type1</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>legal_status</t>
+          <t>type2</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
@@ -507,7 +511,7 @@
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>activities</t>
+          <t>programs_activities</t>
         </is>
       </c>
       <c r="J1" s="4" t="inlineStr">
@@ -532,7 +536,7 @@
       </c>
       <c r="N1" s="4" t="inlineStr">
         <is>
-          <t>partnerships</t>
+          <t>partners</t>
         </is>
       </c>
       <c r="O1" s="4" t="inlineStr">
@@ -547,69 +551,103 @@
       </c>
       <c r="Q1" s="4" t="inlineStr">
         <is>
-          <t>founder</t>
+          <t>founders</t>
         </is>
       </c>
       <c r="R1" s="4" t="inlineStr">
         <is>
-          <t>equipments</t>
+          <t>facilities</t>
         </is>
       </c>
       <c r="S1" s="4" t="inlineStr">
         <is>
+          <t>authority</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>jurisdiction</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>members</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>collections</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>graduates</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>undergraduates</t>
+        </is>
+      </c>
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
           <t>score</t>
         </is>
       </c>
-      <c r="T1" s="4" t="inlineStr">
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>city_id</t>
         </is>
       </c>
-      <c r="U1" s="4" t="inlineStr">
+      <c r="AA1" s="4" t="inlineStr">
         <is>
           <t>numberOfEmployees</t>
         </is>
       </c>
-      <c r="V1" s="4" t="inlineStr">
+      <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>personnel</t>
         </is>
       </c>
-      <c r="W1" s="4" t="inlineStr">
+      <c r="AC1" s="4" t="inlineStr">
         <is>
           <t>numberOfSubsidiaries</t>
         </is>
       </c>
-      <c r="X1" s="4" t="inlineStr">
+      <c r="AD1" s="4" t="inlineStr">
         <is>
           <t>parent_organization_id</t>
         </is>
       </c>
-      <c r="Y1" s="4" t="inlineStr">
+      <c r="AE1" s="4" t="inlineStr">
         <is>
           <t>metadata</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <autoFilter ref="A1:Y1"/>
-  <dataValidations count="5">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
+  <autoFilter ref="A1:AE1"/>
+  <dataValidations count="6">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please select a value from the dropdown list." type="list">
       <formula1>_lists!$B$2:$B$12</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="Please enter a whole number." type="whole" operator="between">
+    <dataValidation sqref="U2:U1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="Please enter a whole number." type="whole" operator="between">
       <formula1>-2147483648</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation sqref="U2:U1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please select a value from the dropdown list." type="list">
-      <formula1>_lists!$A$2:$A$7</formula1>
-    </dataValidation>
-    <dataValidation sqref="V2:V1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="Please enter a whole number." type="whole" operator="between">
+    <dataValidation sqref="Y2:Y1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="Please enter a whole number." type="whole" operator="between">
       <formula1>-2147483648</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation sqref="W2:W1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="Please enter a whole number." type="whole" operator="between">
+    <dataValidation sqref="AA2:AA1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please select a value from the dropdown list." type="list">
+      <formula1>_lists!$A$2:$A$7</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB2:AB1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="Please enter a whole number." type="whole" operator="between">
+      <formula1>-2147483648</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation sqref="AC2:AC1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="Please enter a whole number." type="whole" operator="between">
       <formula1>-2147483648</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>

</xml_diff>